<commit_message>
docs: correct endpoint, table and route counts across the document set
Verified against the source: 17 tables, 62 endpoints, 31 client routes over 27
page modules. These are figures a reviewer will check, so they are now derived
from the code rather than estimated.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/AVSAR_Code_Register_v1.0.xlsx
+++ b/docs/AVSAR_Code_Register_v1.0.xlsx
@@ -1299,7 +1299,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Sixteen tables in portable SQL with foreign keys, unique constraints and indexes.</t>
+          <t>Seventeen tables in portable SQL with foreign keys, unique constraints and indexes.</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>46 endpoints</t>
+          <t>62 endpoints</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">

</xml_diff>